<commit_message>
Changed Remarks to DO NOT Mount
Remarks for SMD Pads and Tag Connect are DO NOT Mount as this is not a purchasable part.
</commit_message>
<xml_diff>
--- a/Documents/Martin_BOM_DigiKey.xlsx
+++ b/Documents/Martin_BOM_DigiKey.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="23628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temporary\MartinS\Martin_Smith\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D920A35-B213-458A-BA7C-A5F9B7DA79E2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="254">
   <si>
     <t>S. No.</t>
   </si>
@@ -94,9 +93,6 @@
     <t>Mouser</t>
   </si>
   <si>
-    <t>not available on digikey</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -782,12 +778,15 @@
   </si>
   <si>
     <t>$7.34/lot (20pieces)</t>
+  </si>
+  <si>
+    <t>DO NOT Mount</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -1368,263 +1367,263 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1727,23 +1726,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1779,23 +1761,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1971,7 +1936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1994,76 +1959,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="31"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="27"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="38" t="s">
-        <v>236</v>
-      </c>
-      <c r="C2" s="66" t="s">
+      <c r="B2" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="C2" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="66" t="s">
+      <c r="D2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="66" t="s">
+      <c r="E2" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="66" t="s">
-        <v>235</v>
-      </c>
-      <c r="H2" s="66" t="s">
+      <c r="G2" s="56" t="s">
+        <v>234</v>
+      </c>
+      <c r="H2" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="66" t="s">
+      <c r="K2" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="66" t="s">
+      <c r="L2" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="66" t="s">
+      <c r="M2" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="66" t="s">
+      <c r="N2" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="66" t="s">
+      <c r="O2" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="67" t="s">
+      <c r="P2" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="68" t="s">
+      <c r="Q2" s="58" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2071,49 +2036,49 @@
       <c r="A3" s="22">
         <v>1</v>
       </c>
-      <c r="B3" s="45" t="s">
-        <v>237</v>
-      </c>
-      <c r="C3" s="69" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="69" t="s">
-        <v>77</v>
-      </c>
-      <c r="E3" s="69" t="s">
-        <v>121</v>
-      </c>
-      <c r="F3" s="69" t="s">
-        <v>149</v>
-      </c>
-      <c r="G3" s="69" t="s">
-        <v>212</v>
-      </c>
-      <c r="H3" s="60"/>
-      <c r="I3" s="69" t="s">
-        <v>183</v>
-      </c>
-      <c r="J3" s="70">
+      <c r="B3" s="107" t="s">
+        <v>236</v>
+      </c>
+      <c r="C3" s="59" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="59" t="s">
+        <v>120</v>
+      </c>
+      <c r="F3" s="59" t="s">
+        <v>148</v>
+      </c>
+      <c r="G3" s="59" t="s">
+        <v>211</v>
+      </c>
+      <c r="H3" s="51"/>
+      <c r="I3" s="59" t="s">
+        <v>182</v>
+      </c>
+      <c r="J3" s="60">
         <v>2</v>
       </c>
-      <c r="K3" s="46">
+      <c r="K3" s="37">
         <f>J3*5</f>
         <v>10</v>
       </c>
-      <c r="L3" s="85" t="s">
+      <c r="L3" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="61">
+      <c r="M3" s="52">
         <v>0.1</v>
       </c>
-      <c r="N3" s="48">
+      <c r="N3" s="39">
         <f>J3*M3</f>
         <v>0.2</v>
       </c>
-      <c r="O3" s="86">
+      <c r="O3" s="76">
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="P3" s="49">
+      <c r="P3" s="40">
         <f>O3*K3</f>
         <v>0.21000000000000002</v>
       </c>
@@ -2123,47 +2088,47 @@
       <c r="A4" s="16">
         <v>2</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="71" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="71" t="s">
-        <v>78</v>
-      </c>
-      <c r="E4" s="71" t="s">
-        <v>122</v>
-      </c>
-      <c r="F4" s="71" t="s">
-        <v>150</v>
-      </c>
-      <c r="G4" s="71" t="s">
-        <v>213</v>
+      <c r="B4" s="108"/>
+      <c r="C4" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="61" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>121</v>
+      </c>
+      <c r="F4" s="61" t="s">
+        <v>149</v>
+      </c>
+      <c r="G4" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="H4" s="10"/>
-      <c r="I4" s="71" t="s">
-        <v>184</v>
-      </c>
-      <c r="J4" s="72">
+      <c r="I4" s="61" t="s">
+        <v>183</v>
+      </c>
+      <c r="J4" s="62">
         <v>6</v>
       </c>
       <c r="K4" s="11">
         <f>J4*5</f>
         <v>30</v>
       </c>
-      <c r="L4" s="87" t="s">
+      <c r="L4" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="88">
+      <c r="M4" s="78">
         <v>0.22</v>
       </c>
-      <c r="N4" s="48">
+      <c r="N4" s="39">
         <f>J4*M4</f>
         <v>1.32</v>
       </c>
       <c r="O4" s="12">
         <v>0.14699999999999999</v>
       </c>
-      <c r="P4" s="49">
+      <c r="P4" s="40">
         <f t="shared" ref="P4:P50" si="0">O4*K4</f>
         <v>4.41</v>
       </c>
@@ -2173,47 +2138,47 @@
       <c r="A5" s="16">
         <v>3</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="71" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="71" t="s">
-        <v>79</v>
-      </c>
-      <c r="E5" s="71" t="s">
-        <v>123</v>
-      </c>
-      <c r="F5" s="71" t="s">
-        <v>151</v>
-      </c>
-      <c r="G5" s="71" t="s">
-        <v>213</v>
+      <c r="B5" s="108"/>
+      <c r="C5" s="61" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="61" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" s="61" t="s">
+        <v>150</v>
+      </c>
+      <c r="G5" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="H5" s="13"/>
-      <c r="I5" s="71" t="s">
-        <v>185</v>
-      </c>
-      <c r="J5" s="72">
+      <c r="I5" s="61" t="s">
+        <v>184</v>
+      </c>
+      <c r="J5" s="62">
         <v>2</v>
       </c>
       <c r="K5" s="11">
         <f t="shared" ref="K5:K50" si="1">J5*5</f>
         <v>10</v>
       </c>
-      <c r="L5" s="87" t="s">
+      <c r="L5" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M5" s="14">
         <v>0.52</v>
       </c>
-      <c r="N5" s="48">
-        <f t="shared" ref="N4:N50" si="2">J5*M5</f>
+      <c r="N5" s="39">
+        <f t="shared" ref="N5:N50" si="2">J5*M5</f>
         <v>1.04</v>
       </c>
       <c r="O5" s="14">
         <v>0.36499999999999999</v>
       </c>
-      <c r="P5" s="49">
+      <c r="P5" s="40">
         <f t="shared" si="0"/>
         <v>3.65</v>
       </c>
@@ -2223,47 +2188,47 @@
       <c r="A6" s="16">
         <v>4</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="71" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="71" t="s">
-        <v>80</v>
-      </c>
-      <c r="E6" s="71" t="s">
-        <v>121</v>
-      </c>
-      <c r="F6" s="71" t="s">
-        <v>152</v>
-      </c>
-      <c r="G6" s="71" t="s">
-        <v>213</v>
+      <c r="B6" s="108"/>
+      <c r="C6" s="61" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="61" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="61" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="H6" s="10"/>
-      <c r="I6" s="71" t="s">
-        <v>186</v>
-      </c>
-      <c r="J6" s="72">
+      <c r="I6" s="61" t="s">
+        <v>185</v>
+      </c>
+      <c r="J6" s="62">
         <v>11</v>
       </c>
       <c r="K6" s="11">
         <f>J6*5</f>
         <v>55</v>
       </c>
-      <c r="L6" s="87" t="s">
+      <c r="L6" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M6" s="12">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="N6" s="48">
+      <c r="N6" s="39">
         <f t="shared" si="2"/>
         <v>0.56099999999999994</v>
       </c>
       <c r="O6" s="12">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="P6" s="49">
+      <c r="P6" s="40">
         <f t="shared" si="0"/>
         <v>1.5289999999999999</v>
       </c>
@@ -2273,47 +2238,47 @@
       <c r="A7" s="16">
         <v>5</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="71" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="71" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" s="71" t="s">
-        <v>121</v>
-      </c>
-      <c r="F7" s="71" t="s">
-        <v>153</v>
-      </c>
-      <c r="G7" s="71" t="s">
-        <v>214</v>
+      <c r="B7" s="108"/>
+      <c r="C7" s="61" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="61" t="s">
+        <v>120</v>
+      </c>
+      <c r="F7" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="G7" s="61" t="s">
+        <v>213</v>
       </c>
       <c r="H7" s="13"/>
-      <c r="I7" s="71" t="s">
-        <v>187</v>
-      </c>
-      <c r="J7" s="72">
+      <c r="I7" s="61" t="s">
+        <v>186</v>
+      </c>
+      <c r="J7" s="62">
         <v>9</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="L7" s="87" t="s">
+      <c r="L7" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M7" s="15">
         <v>0.28000000000000003</v>
       </c>
-      <c r="N7" s="48">
+      <c r="N7" s="39">
         <f t="shared" si="2"/>
         <v>2.5200000000000005</v>
       </c>
       <c r="O7" s="15">
         <v>0.189</v>
       </c>
-      <c r="P7" s="49">
+      <c r="P7" s="40">
         <f t="shared" si="0"/>
         <v>8.5050000000000008</v>
       </c>
@@ -2323,47 +2288,47 @@
       <c r="A8" s="16">
         <v>6</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="71" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="71" t="s">
-        <v>82</v>
-      </c>
-      <c r="E8" s="71" t="s">
-        <v>124</v>
-      </c>
-      <c r="F8" s="71" t="s">
-        <v>154</v>
-      </c>
-      <c r="G8" s="71" t="s">
-        <v>213</v>
+      <c r="B8" s="108"/>
+      <c r="C8" s="61" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="E8" s="61" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" s="61" t="s">
+        <v>153</v>
+      </c>
+      <c r="G8" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="H8" s="10"/>
-      <c r="I8" s="71" t="s">
-        <v>188</v>
-      </c>
-      <c r="J8" s="72">
+      <c r="I8" s="61" t="s">
+        <v>187</v>
+      </c>
+      <c r="J8" s="62">
         <v>1</v>
       </c>
       <c r="K8" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L8" s="87" t="s">
+      <c r="L8" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M8" s="12">
         <v>0.1</v>
       </c>
-      <c r="N8" s="48">
+      <c r="N8" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O8" s="12">
         <v>0.1</v>
       </c>
-      <c r="P8" s="49">
+      <c r="P8" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -2373,47 +2338,47 @@
       <c r="A9" s="16">
         <v>7</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="71" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="71" t="s">
-        <v>83</v>
-      </c>
-      <c r="E9" s="71" t="s">
-        <v>122</v>
-      </c>
-      <c r="F9" s="71" t="s">
-        <v>155</v>
-      </c>
-      <c r="G9" s="71" t="s">
-        <v>215</v>
+      <c r="B9" s="108"/>
+      <c r="C9" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="61" t="s">
+        <v>121</v>
+      </c>
+      <c r="F9" s="61" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="61" t="s">
+        <v>214</v>
       </c>
       <c r="H9" s="23"/>
-      <c r="I9" s="71" t="s">
-        <v>189</v>
-      </c>
-      <c r="J9" s="72">
+      <c r="I9" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="J9" s="62">
         <v>1</v>
       </c>
       <c r="K9" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L9" s="87" t="s">
+      <c r="L9" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M9" s="12">
         <v>0.32</v>
       </c>
-      <c r="N9" s="48">
+      <c r="N9" s="39">
         <f t="shared" si="2"/>
         <v>0.32</v>
       </c>
       <c r="O9" s="12">
         <v>0.32</v>
       </c>
-      <c r="P9" s="49">
+      <c r="P9" s="40">
         <f t="shared" si="0"/>
         <v>1.6</v>
       </c>
@@ -2423,47 +2388,47 @@
       <c r="A10" s="16">
         <v>8</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="71" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="71" t="s">
-        <v>84</v>
-      </c>
-      <c r="E10" s="71" t="s">
-        <v>123</v>
-      </c>
-      <c r="F10" s="71" t="s">
-        <v>156</v>
-      </c>
-      <c r="G10" s="71" t="s">
-        <v>213</v>
+      <c r="B10" s="108"/>
+      <c r="C10" s="61" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="61" t="s">
+        <v>122</v>
+      </c>
+      <c r="F10" s="61" t="s">
+        <v>155</v>
+      </c>
+      <c r="G10" s="61" t="s">
+        <v>212</v>
       </c>
       <c r="H10" s="13"/>
-      <c r="I10" s="71" t="s">
-        <v>190</v>
-      </c>
-      <c r="J10" s="72">
+      <c r="I10" s="61" t="s">
+        <v>189</v>
+      </c>
+      <c r="J10" s="62">
         <v>1</v>
       </c>
       <c r="K10" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L10" s="87" t="s">
+      <c r="L10" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M10" s="14">
         <v>0.32</v>
       </c>
-      <c r="N10" s="48">
+      <c r="N10" s="39">
         <f t="shared" si="2"/>
         <v>0.32</v>
       </c>
       <c r="O10" s="14">
         <v>0.32</v>
       </c>
-      <c r="P10" s="49">
+      <c r="P10" s="40">
         <f t="shared" si="0"/>
         <v>1.6</v>
       </c>
@@ -2473,47 +2438,47 @@
       <c r="A11" s="16">
         <v>9</v>
       </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="71" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="71" t="s">
-        <v>85</v>
-      </c>
-      <c r="E11" s="71" t="s">
-        <v>121</v>
-      </c>
-      <c r="F11" s="71" t="s">
-        <v>157</v>
-      </c>
-      <c r="G11" s="71" t="s">
-        <v>216</v>
+      <c r="B11" s="108"/>
+      <c r="C11" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="61" t="s">
+        <v>120</v>
+      </c>
+      <c r="F11" s="61" t="s">
+        <v>156</v>
+      </c>
+      <c r="G11" s="61" t="s">
+        <v>215</v>
       </c>
       <c r="H11" s="10"/>
-      <c r="I11" s="71" t="s">
-        <v>191</v>
-      </c>
-      <c r="J11" s="72">
+      <c r="I11" s="61" t="s">
+        <v>190</v>
+      </c>
+      <c r="J11" s="62">
         <v>1</v>
       </c>
       <c r="K11" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L11" s="87" t="s">
+      <c r="L11" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="M11" s="89">
+      <c r="M11" s="79">
         <v>0.1</v>
       </c>
-      <c r="N11" s="48">
+      <c r="N11" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O11" s="12">
         <v>0.1</v>
       </c>
-      <c r="P11" s="49">
+      <c r="P11" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -2523,47 +2488,47 @@
       <c r="A12" s="16">
         <v>10</v>
       </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="71" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="71" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="71" t="s">
-        <v>125</v>
-      </c>
-      <c r="F12" s="71" t="s">
-        <v>158</v>
-      </c>
-      <c r="G12" s="71" t="s">
-        <v>217</v>
+      <c r="B12" s="108"/>
+      <c r="C12" s="61" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>124</v>
+      </c>
+      <c r="F12" s="61" t="s">
+        <v>157</v>
+      </c>
+      <c r="G12" s="61" t="s">
+        <v>216</v>
       </c>
       <c r="H12" s="13"/>
-      <c r="I12" s="71" t="s">
-        <v>192</v>
-      </c>
-      <c r="J12" s="72">
+      <c r="I12" s="61" t="s">
+        <v>191</v>
+      </c>
+      <c r="J12" s="62">
         <v>2</v>
       </c>
       <c r="K12" s="11">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L12" s="87" t="s">
+      <c r="L12" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M12" s="12">
         <v>0.47</v>
       </c>
-      <c r="N12" s="48">
+      <c r="N12" s="39">
         <f t="shared" si="2"/>
         <v>0.94</v>
       </c>
       <c r="O12" s="12">
         <v>0.33100000000000002</v>
       </c>
-      <c r="P12" s="49">
+      <c r="P12" s="40">
         <f t="shared" si="0"/>
         <v>3.31</v>
       </c>
@@ -2573,151 +2538,151 @@
       <c r="A13" s="16">
         <v>11</v>
       </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="71" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="71" t="s">
-        <v>87</v>
-      </c>
-      <c r="E13" s="71" t="s">
-        <v>122</v>
-      </c>
-      <c r="F13" s="71" t="s">
-        <v>159</v>
-      </c>
-      <c r="G13" s="71" t="s">
-        <v>218</v>
+      <c r="B13" s="108"/>
+      <c r="C13" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="61" t="s">
+        <v>121</v>
+      </c>
+      <c r="F13" s="61" t="s">
+        <v>158</v>
+      </c>
+      <c r="G13" s="61" t="s">
+        <v>217</v>
       </c>
       <c r="H13" s="10"/>
-      <c r="I13" s="71" t="s">
-        <v>193</v>
-      </c>
-      <c r="J13" s="72">
+      <c r="I13" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="J13" s="62">
         <v>1</v>
       </c>
       <c r="K13" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L13" s="87" t="s">
+      <c r="L13" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M13" s="12">
         <v>0.1</v>
       </c>
-      <c r="N13" s="48">
+      <c r="N13" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O13" s="12">
         <v>0.1</v>
       </c>
-      <c r="P13" s="49">
+      <c r="P13" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
       <c r="Q13" s="9"/>
     </row>
     <row r="14" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="32">
+      <c r="A14" s="28">
         <v>12</v>
       </c>
-      <c r="B14" s="90" t="s">
+      <c r="B14" s="80" t="s">
+        <v>245</v>
+      </c>
+      <c r="C14" s="63" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="63" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="F14" s="63" t="s">
         <v>246</v>
       </c>
-      <c r="C14" s="73" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="73" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" s="73" t="s">
-        <v>126</v>
-      </c>
-      <c r="F14" s="73" t="s">
-        <v>247</v>
-      </c>
-      <c r="G14" s="73" t="s">
-        <v>219</v>
+      <c r="G14" s="63" t="s">
+        <v>218</v>
       </c>
       <c r="H14" s="24"/>
-      <c r="I14" s="73" t="s">
-        <v>160</v>
-      </c>
-      <c r="J14" s="74">
+      <c r="I14" s="63" t="s">
+        <v>159</v>
+      </c>
+      <c r="J14" s="64">
         <v>2</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L14" s="91" t="s">
+      <c r="L14" s="81" t="s">
         <v>14</v>
       </c>
       <c r="M14" s="20">
         <v>0.53</v>
       </c>
-      <c r="N14" s="48">
+      <c r="N14" s="39">
         <f t="shared" si="2"/>
         <v>1.06</v>
       </c>
       <c r="O14" s="20">
         <v>0.45400000000000001</v>
       </c>
-      <c r="P14" s="49">
+      <c r="P14" s="40">
         <f t="shared" si="0"/>
         <v>4.54</v>
       </c>
-      <c r="Q14" s="34"/>
+      <c r="Q14" s="30"/>
     </row>
     <row r="15" spans="1:17" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="22">
         <v>13</v>
       </c>
-      <c r="B15" s="45" t="s">
-        <v>238</v>
-      </c>
-      <c r="C15" s="69" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="69" t="s">
-        <v>89</v>
-      </c>
-      <c r="E15" s="69" t="s">
-        <v>127</v>
-      </c>
-      <c r="F15" s="69" t="s">
-        <v>127</v>
-      </c>
-      <c r="G15" s="69" t="s">
-        <v>220</v>
-      </c>
-      <c r="H15" s="60"/>
-      <c r="I15" s="69" t="s">
-        <v>127</v>
-      </c>
-      <c r="J15" s="70">
+      <c r="B15" s="107" t="s">
+        <v>237</v>
+      </c>
+      <c r="C15" s="59" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="F15" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="G15" s="59" t="s">
+        <v>219</v>
+      </c>
+      <c r="H15" s="51"/>
+      <c r="I15" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="J15" s="60">
         <v>1</v>
       </c>
-      <c r="K15" s="46">
+      <c r="K15" s="37">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L15" s="85" t="s">
+      <c r="L15" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="M15" s="61">
+      <c r="M15" s="52">
         <v>0.19</v>
       </c>
-      <c r="N15" s="48">
+      <c r="N15" s="39">
         <f t="shared" si="2"/>
         <v>0.19</v>
       </c>
-      <c r="O15" s="61">
+      <c r="O15" s="52">
         <v>0.19</v>
       </c>
-      <c r="P15" s="49">
+      <c r="P15" s="40">
         <f t="shared" si="0"/>
         <v>0.95</v>
       </c>
@@ -2727,497 +2692,499 @@
       <c r="A16" s="16">
         <v>14</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="95" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="95" t="s">
-        <v>90</v>
-      </c>
-      <c r="E16" s="95" t="s">
-        <v>128</v>
-      </c>
-      <c r="F16" s="95" t="s">
-        <v>128</v>
-      </c>
-      <c r="G16" s="96"/>
-      <c r="H16" s="97"/>
-      <c r="I16" s="95" t="s">
-        <v>194</v>
-      </c>
-      <c r="J16" s="96">
+      <c r="B16" s="108"/>
+      <c r="C16" s="85" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="85" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="85" t="s">
+        <v>127</v>
+      </c>
+      <c r="F16" s="85" t="s">
+        <v>127</v>
+      </c>
+      <c r="G16" s="86"/>
+      <c r="H16" s="87"/>
+      <c r="I16" s="85" t="s">
+        <v>193</v>
+      </c>
+      <c r="J16" s="86">
         <v>1</v>
       </c>
-      <c r="K16" s="98">
+      <c r="K16" s="88">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L16" s="99"/>
-      <c r="M16" s="100"/>
-      <c r="N16" s="101">
+      <c r="L16" s="89"/>
+      <c r="M16" s="90"/>
+      <c r="N16" s="91">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O16" s="100"/>
-      <c r="P16" s="102">
+      <c r="O16" s="90"/>
+      <c r="P16" s="92">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Q16" s="103" t="s">
-        <v>24</v>
+      <c r="Q16" s="93" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="16">
         <v>15</v>
       </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="95" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="95" t="s">
-        <v>91</v>
-      </c>
-      <c r="E17" s="95" t="s">
-        <v>129</v>
-      </c>
-      <c r="F17" s="95" t="s">
-        <v>129</v>
-      </c>
-      <c r="G17" s="95" t="s">
-        <v>221</v>
-      </c>
-      <c r="H17" s="97"/>
-      <c r="I17" s="95" t="s">
-        <v>129</v>
-      </c>
-      <c r="J17" s="96">
+      <c r="B17" s="108"/>
+      <c r="C17" s="85" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="85" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="85" t="s">
+        <v>128</v>
+      </c>
+      <c r="F17" s="85" t="s">
+        <v>128</v>
+      </c>
+      <c r="G17" s="85" t="s">
+        <v>220</v>
+      </c>
+      <c r="H17" s="87"/>
+      <c r="I17" s="85" t="s">
+        <v>128</v>
+      </c>
+      <c r="J17" s="86">
         <v>1</v>
       </c>
-      <c r="K17" s="98">
+      <c r="K17" s="88">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L17" s="99"/>
-      <c r="M17" s="100"/>
-      <c r="N17" s="101">
+      <c r="L17" s="89"/>
+      <c r="M17" s="90"/>
+      <c r="N17" s="91">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O17" s="100"/>
-      <c r="P17" s="102">
+      <c r="O17" s="90"/>
+      <c r="P17" s="92">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Q17" s="103"/>
+      <c r="Q17" s="93" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="18" spans="1:17" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="16">
         <v>16</v>
       </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="71" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="71" t="s">
-        <v>92</v>
-      </c>
-      <c r="E18" s="71" t="s">
-        <v>130</v>
-      </c>
-      <c r="F18" s="71" t="s">
-        <v>130</v>
-      </c>
-      <c r="G18" s="71" t="s">
-        <v>220</v>
+      <c r="B18" s="108"/>
+      <c r="C18" s="61" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="61" t="s">
+        <v>129</v>
+      </c>
+      <c r="F18" s="61" t="s">
+        <v>129</v>
+      </c>
+      <c r="G18" s="61" t="s">
+        <v>219</v>
       </c>
       <c r="H18" s="23"/>
-      <c r="I18" s="71" t="s">
-        <v>130</v>
-      </c>
-      <c r="J18" s="72">
+      <c r="I18" s="61" t="s">
+        <v>129</v>
+      </c>
+      <c r="J18" s="62">
         <v>1</v>
       </c>
       <c r="K18" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L18" s="87" t="s">
+      <c r="L18" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M18" s="15">
         <v>0.24</v>
       </c>
-      <c r="N18" s="48">
+      <c r="N18" s="39">
         <f t="shared" si="2"/>
         <v>0.24</v>
       </c>
       <c r="O18" s="14">
         <v>0.24</v>
       </c>
-      <c r="P18" s="49">
+      <c r="P18" s="40">
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
       <c r="Q18" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="32">
+      <c r="A19" s="28">
         <v>17</v>
       </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="73" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="73" t="s">
-        <v>93</v>
-      </c>
-      <c r="E19" s="73" t="s">
-        <v>131</v>
-      </c>
-      <c r="F19" s="73" t="s">
-        <v>131</v>
-      </c>
-      <c r="G19" s="73" t="s">
-        <v>222</v>
+      <c r="B19" s="109"/>
+      <c r="C19" s="63" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="63" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" s="63" t="s">
+        <v>130</v>
+      </c>
+      <c r="F19" s="63" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" s="63" t="s">
+        <v>221</v>
       </c>
       <c r="H19" s="17"/>
-      <c r="I19" s="73" t="s">
-        <v>131</v>
-      </c>
-      <c r="J19" s="74">
+      <c r="I19" s="63" t="s">
+        <v>130</v>
+      </c>
+      <c r="J19" s="64">
         <v>1</v>
       </c>
       <c r="K19" s="18">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L19" s="91" t="s">
+      <c r="L19" s="81" t="s">
         <v>14</v>
       </c>
-      <c r="M19" s="64">
+      <c r="M19" s="54">
         <v>1.19</v>
       </c>
-      <c r="N19" s="48">
+      <c r="N19" s="39">
         <f t="shared" si="2"/>
         <v>1.19</v>
       </c>
-      <c r="O19" s="64">
+      <c r="O19" s="54">
         <v>1.19</v>
       </c>
-      <c r="P19" s="49">
+      <c r="P19" s="40">
         <f t="shared" si="0"/>
         <v>5.9499999999999993</v>
       </c>
-      <c r="Q19" s="65" t="s">
-        <v>26</v>
+      <c r="Q19" s="55" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="22">
         <v>18</v>
       </c>
-      <c r="B20" s="45" t="s">
-        <v>239</v>
-      </c>
-      <c r="C20" s="69" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="69" t="s">
-        <v>94</v>
-      </c>
-      <c r="E20" s="69" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20" s="69" t="s">
-        <v>132</v>
-      </c>
-      <c r="G20" s="69" t="s">
-        <v>223</v>
-      </c>
-      <c r="H20" s="60"/>
-      <c r="I20" s="69" t="s">
-        <v>195</v>
-      </c>
-      <c r="J20" s="70">
+      <c r="B20" s="107" t="s">
+        <v>238</v>
+      </c>
+      <c r="C20" s="59" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="59" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="59" t="s">
+        <v>131</v>
+      </c>
+      <c r="F20" s="59" t="s">
+        <v>131</v>
+      </c>
+      <c r="G20" s="59" t="s">
+        <v>222</v>
+      </c>
+      <c r="H20" s="51"/>
+      <c r="I20" s="59" t="s">
+        <v>194</v>
+      </c>
+      <c r="J20" s="60">
         <v>1</v>
       </c>
-      <c r="K20" s="46">
+      <c r="K20" s="37">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L20" s="85" t="s">
+      <c r="L20" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="M20" s="61">
+      <c r="M20" s="52">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N20" s="48">
+      <c r="N20" s="39">
         <f t="shared" si="2"/>
         <v>0.55000000000000004</v>
       </c>
-      <c r="O20" s="61">
+      <c r="O20" s="52">
         <v>0.55000000000000004</v>
       </c>
-      <c r="P20" s="49">
+      <c r="P20" s="40">
         <f t="shared" si="0"/>
         <v>2.75</v>
       </c>
-      <c r="Q20" s="62"/>
+      <c r="Q20" s="53"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16">
         <v>19</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="D21" s="71" t="s">
-        <v>95</v>
-      </c>
-      <c r="E21" s="71" t="s">
-        <v>133</v>
-      </c>
-      <c r="F21" s="71" t="s">
-        <v>133</v>
-      </c>
-      <c r="G21" s="71" t="s">
-        <v>223</v>
+      <c r="B21" s="110"/>
+      <c r="C21" s="61" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="61" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="F21" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="G21" s="61" t="s">
+        <v>222</v>
       </c>
       <c r="H21" s="10"/>
-      <c r="I21" s="71" t="s">
-        <v>196</v>
-      </c>
-      <c r="J21" s="72">
+      <c r="I21" s="61" t="s">
+        <v>195</v>
+      </c>
+      <c r="J21" s="62">
         <v>1</v>
       </c>
       <c r="K21" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L21" s="87" t="s">
+      <c r="L21" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M21" s="12">
         <v>0.92</v>
       </c>
-      <c r="N21" s="48">
+      <c r="N21" s="39">
         <f t="shared" si="2"/>
         <v>0.92</v>
       </c>
       <c r="O21" s="12">
         <v>0.92</v>
       </c>
-      <c r="P21" s="49">
+      <c r="P21" s="40">
         <f t="shared" si="0"/>
         <v>4.6000000000000005</v>
       </c>
       <c r="Q21" s="9"/>
     </row>
     <row r="22" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="32">
+      <c r="A22" s="28">
         <v>20</v>
       </c>
-      <c r="B22" s="63"/>
-      <c r="C22" s="73" t="s">
-        <v>49</v>
-      </c>
-      <c r="D22" s="73" t="s">
-        <v>96</v>
-      </c>
-      <c r="E22" s="73" t="s">
-        <v>134</v>
-      </c>
-      <c r="F22" s="73" t="s">
-        <v>161</v>
-      </c>
-      <c r="G22" s="73" t="s">
-        <v>215</v>
-      </c>
-      <c r="H22" s="79"/>
-      <c r="I22" s="73" t="s">
-        <v>197</v>
-      </c>
-      <c r="J22" s="74">
+      <c r="B22" s="111"/>
+      <c r="C22" s="63" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" s="63" t="s">
+        <v>133</v>
+      </c>
+      <c r="F22" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="G22" s="63" t="s">
+        <v>214</v>
+      </c>
+      <c r="H22" s="69"/>
+      <c r="I22" s="63" t="s">
+        <v>196</v>
+      </c>
+      <c r="J22" s="64">
         <v>1</v>
       </c>
       <c r="K22" s="18">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L22" s="91" t="s">
+      <c r="L22" s="81" t="s">
         <v>14</v>
       </c>
       <c r="M22" s="20">
         <v>0.38</v>
       </c>
-      <c r="N22" s="48">
+      <c r="N22" s="39">
         <f t="shared" si="2"/>
         <v>0.38</v>
       </c>
       <c r="O22" s="20">
         <v>0.38</v>
       </c>
-      <c r="P22" s="49">
+      <c r="P22" s="40">
         <f t="shared" si="0"/>
         <v>1.9</v>
       </c>
-      <c r="Q22" s="34"/>
+      <c r="Q22" s="30"/>
     </row>
     <row r="23" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="50">
+      <c r="A23" s="41">
         <v>21</v>
       </c>
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="75" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="E23" s="75" t="s">
-        <v>135</v>
-      </c>
-      <c r="F23" s="75" t="s">
-        <v>162</v>
-      </c>
-      <c r="G23" s="75" t="s">
-        <v>224</v>
-      </c>
-      <c r="H23" s="80"/>
-      <c r="I23" s="75" t="s">
-        <v>162</v>
-      </c>
-      <c r="J23" s="76">
+      <c r="C23" s="65" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="65" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="65" t="s">
+        <v>134</v>
+      </c>
+      <c r="F23" s="65" t="s">
+        <v>161</v>
+      </c>
+      <c r="G23" s="65" t="s">
+        <v>223</v>
+      </c>
+      <c r="H23" s="70"/>
+      <c r="I23" s="65" t="s">
+        <v>161</v>
+      </c>
+      <c r="J23" s="66">
         <v>1</v>
       </c>
-      <c r="K23" s="52">
+      <c r="K23" s="43">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L23" s="92" t="s">
+      <c r="L23" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="M23" s="53">
+      <c r="M23" s="44">
         <v>0.34</v>
       </c>
-      <c r="N23" s="48">
+      <c r="N23" s="39">
         <f t="shared" si="2"/>
         <v>0.34</v>
       </c>
-      <c r="O23" s="53">
+      <c r="O23" s="44">
         <v>0.34</v>
       </c>
-      <c r="P23" s="49">
+      <c r="P23" s="40">
         <f t="shared" si="0"/>
         <v>1.7000000000000002</v>
       </c>
-      <c r="Q23" s="54"/>
+      <c r="Q23" s="45"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="55">
+      <c r="A24" s="46">
         <v>22</v>
       </c>
-      <c r="B24" s="56" t="s">
-        <v>240</v>
-      </c>
-      <c r="C24" s="77" t="s">
-        <v>51</v>
-      </c>
-      <c r="D24" s="77" t="s">
-        <v>98</v>
-      </c>
-      <c r="E24" s="77" t="s">
-        <v>136</v>
-      </c>
-      <c r="F24" s="77" t="s">
-        <v>163</v>
-      </c>
-      <c r="G24" s="77" t="s">
-        <v>225</v>
-      </c>
-      <c r="H24" s="81"/>
-      <c r="I24" s="77" t="s">
-        <v>163</v>
-      </c>
-      <c r="J24" s="78">
+      <c r="B24" s="47" t="s">
+        <v>239</v>
+      </c>
+      <c r="C24" s="67" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="67" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24" s="67" t="s">
+        <v>135</v>
+      </c>
+      <c r="F24" s="67" t="s">
+        <v>162</v>
+      </c>
+      <c r="G24" s="67" t="s">
+        <v>224</v>
+      </c>
+      <c r="H24" s="71"/>
+      <c r="I24" s="67" t="s">
+        <v>162</v>
+      </c>
+      <c r="J24" s="68">
         <v>1</v>
       </c>
-      <c r="K24" s="57">
+      <c r="K24" s="48">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L24" s="93" t="s">
+      <c r="L24" s="83" t="s">
         <v>14</v>
       </c>
-      <c r="M24" s="58">
+      <c r="M24" s="49">
         <v>0.41</v>
       </c>
-      <c r="N24" s="48">
+      <c r="N24" s="39">
         <f t="shared" si="2"/>
         <v>0.41</v>
       </c>
-      <c r="O24" s="94">
+      <c r="O24" s="84">
         <v>0.41</v>
       </c>
-      <c r="P24" s="49">
+      <c r="P24" s="40">
         <f t="shared" si="0"/>
         <v>2.0499999999999998</v>
       </c>
-      <c r="Q24" s="59"/>
+      <c r="Q24" s="50"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="22">
         <v>23</v>
       </c>
-      <c r="B25" s="45" t="s">
-        <v>241</v>
-      </c>
-      <c r="C25" s="69" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="69" t="s">
-        <v>99</v>
-      </c>
-      <c r="E25" s="69" t="s">
-        <v>137</v>
-      </c>
-      <c r="F25" s="69" t="s">
-        <v>164</v>
-      </c>
-      <c r="G25" s="69" t="s">
-        <v>226</v>
-      </c>
-      <c r="H25" s="82"/>
-      <c r="I25" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="J25" s="70">
+      <c r="B25" s="107" t="s">
+        <v>240</v>
+      </c>
+      <c r="C25" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="59" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="F25" s="59" t="s">
+        <v>163</v>
+      </c>
+      <c r="G25" s="59" t="s">
+        <v>225</v>
+      </c>
+      <c r="H25" s="72"/>
+      <c r="I25" s="59" t="s">
+        <v>197</v>
+      </c>
+      <c r="J25" s="60">
         <v>2</v>
       </c>
-      <c r="K25" s="46">
+      <c r="K25" s="37">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L25" s="85" t="s">
+      <c r="L25" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="M25" s="47">
+      <c r="M25" s="38">
         <v>0.1</v>
       </c>
-      <c r="N25" s="48">
+      <c r="N25" s="39">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
-      <c r="O25" s="47">
+      <c r="O25" s="38">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="P25" s="49">
+      <c r="P25" s="40">
         <f t="shared" si="0"/>
         <v>0.26</v>
       </c>
@@ -3227,47 +3194,47 @@
       <c r="A26" s="16">
         <v>24</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="71" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="71" t="s">
-        <v>100</v>
-      </c>
-      <c r="E26" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F26" s="71" t="s">
-        <v>165</v>
-      </c>
-      <c r="G26" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H26" s="83"/>
-      <c r="I26" s="71" t="s">
-        <v>199</v>
-      </c>
-      <c r="J26" s="72">
+      <c r="B26" s="108"/>
+      <c r="C26" s="61" t="s">
+        <v>52</v>
+      </c>
+      <c r="D26" s="61" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F26" s="61" t="s">
+        <v>164</v>
+      </c>
+      <c r="G26" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H26" s="73"/>
+      <c r="I26" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="J26" s="62">
         <v>1</v>
       </c>
       <c r="K26" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L26" s="87" t="s">
+      <c r="L26" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M26" s="12">
         <v>0.1</v>
       </c>
-      <c r="N26" s="48">
+      <c r="N26" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O26" s="12">
         <v>0.1</v>
       </c>
-      <c r="P26" s="49">
+      <c r="P26" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -3277,47 +3244,47 @@
       <c r="A27" s="16">
         <v>25</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="71" t="s">
-        <v>54</v>
-      </c>
-      <c r="D27" s="71" t="s">
+      <c r="B27" s="108"/>
+      <c r="C27" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F27" s="71" t="s">
-        <v>166</v>
-      </c>
-      <c r="G27" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H27" s="83"/>
-      <c r="I27" s="71" t="s">
-        <v>200</v>
-      </c>
-      <c r="J27" s="72">
+      <c r="E27" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F27" s="61" t="s">
+        <v>165</v>
+      </c>
+      <c r="G27" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H27" s="73"/>
+      <c r="I27" s="61" t="s">
+        <v>199</v>
+      </c>
+      <c r="J27" s="62">
         <v>1</v>
       </c>
       <c r="K27" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L27" s="87" t="s">
+      <c r="L27" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M27" s="12">
         <v>0.1</v>
       </c>
-      <c r="N27" s="48">
+      <c r="N27" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O27" s="12">
         <v>0.1</v>
       </c>
-      <c r="P27" s="49">
+      <c r="P27" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -3327,47 +3294,47 @@
       <c r="A28" s="16">
         <v>26</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="71" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28" s="71" t="s">
-        <v>101</v>
-      </c>
-      <c r="E28" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F28" s="71" t="s">
-        <v>167</v>
-      </c>
-      <c r="G28" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H28" s="83"/>
-      <c r="I28" s="71" t="s">
-        <v>201</v>
-      </c>
-      <c r="J28" s="72">
+      <c r="B28" s="108"/>
+      <c r="C28" s="61" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" s="61" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F28" s="61" t="s">
+        <v>166</v>
+      </c>
+      <c r="G28" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H28" s="73"/>
+      <c r="I28" s="61" t="s">
+        <v>200</v>
+      </c>
+      <c r="J28" s="62">
         <v>1</v>
       </c>
       <c r="K28" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L28" s="87" t="s">
+      <c r="L28" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M28" s="12">
         <v>0.1</v>
       </c>
-      <c r="N28" s="48">
+      <c r="N28" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O28" s="12">
         <v>0.1</v>
       </c>
-      <c r="P28" s="49">
+      <c r="P28" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -3377,47 +3344,47 @@
       <c r="A29" s="16">
         <v>27</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="71" t="s">
-        <v>56</v>
-      </c>
-      <c r="D29" s="71" t="s">
+      <c r="B29" s="108"/>
+      <c r="C29" s="61" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="E29" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F29" s="71" t="s">
-        <v>168</v>
-      </c>
-      <c r="G29" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H29" s="83"/>
-      <c r="I29" s="71" t="s">
-        <v>202</v>
-      </c>
-      <c r="J29" s="72">
+      <c r="E29" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" s="61" t="s">
+        <v>167</v>
+      </c>
+      <c r="G29" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H29" s="73"/>
+      <c r="I29" s="61" t="s">
+        <v>201</v>
+      </c>
+      <c r="J29" s="62">
         <v>1</v>
       </c>
       <c r="K29" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L29" s="87" t="s">
+      <c r="L29" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M29" s="12">
         <v>0.1</v>
       </c>
-      <c r="N29" s="48">
+      <c r="N29" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O29" s="12">
         <v>0.1</v>
       </c>
-      <c r="P29" s="49">
+      <c r="P29" s="40">
         <f>O29*K29</f>
         <v>0.5</v>
       </c>
@@ -3427,47 +3394,47 @@
       <c r="A30" s="16">
         <v>28</v>
       </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="71" t="s">
-        <v>57</v>
-      </c>
-      <c r="D30" s="71" t="s">
-        <v>102</v>
-      </c>
-      <c r="E30" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F30" s="71" t="s">
-        <v>169</v>
-      </c>
-      <c r="G30" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H30" s="83"/>
-      <c r="I30" s="71" t="s">
-        <v>27</v>
-      </c>
-      <c r="J30" s="72">
+      <c r="B30" s="108"/>
+      <c r="C30" s="61" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="61" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F30" s="61" t="s">
+        <v>168</v>
+      </c>
+      <c r="G30" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H30" s="73"/>
+      <c r="I30" s="61" t="s">
+        <v>26</v>
+      </c>
+      <c r="J30" s="62">
         <v>1</v>
       </c>
       <c r="K30" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L30" s="87" t="s">
+      <c r="L30" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M30" s="12">
         <v>0.1</v>
       </c>
-      <c r="N30" s="48">
+      <c r="N30" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O30" s="12">
         <v>0.1</v>
       </c>
-      <c r="P30" s="49">
+      <c r="P30" s="40">
         <f>O30*K30</f>
         <v>0.5</v>
       </c>
@@ -3477,47 +3444,47 @@
       <c r="A31" s="16">
         <v>29</v>
       </c>
-      <c r="B31" s="37"/>
-      <c r="C31" s="71" t="s">
-        <v>58</v>
-      </c>
-      <c r="D31" s="71" t="s">
-        <v>103</v>
-      </c>
-      <c r="E31" s="71" t="s">
-        <v>138</v>
-      </c>
-      <c r="F31" s="71" t="s">
-        <v>170</v>
-      </c>
-      <c r="G31" s="71" t="s">
-        <v>227</v>
-      </c>
-      <c r="H31" s="83"/>
-      <c r="I31" s="71" t="s">
-        <v>170</v>
-      </c>
-      <c r="J31" s="72">
+      <c r="B31" s="108"/>
+      <c r="C31" s="61" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="61" t="s">
+        <v>102</v>
+      </c>
+      <c r="E31" s="61" t="s">
+        <v>137</v>
+      </c>
+      <c r="F31" s="61" t="s">
+        <v>169</v>
+      </c>
+      <c r="G31" s="61" t="s">
+        <v>226</v>
+      </c>
+      <c r="H31" s="73"/>
+      <c r="I31" s="61" t="s">
+        <v>169</v>
+      </c>
+      <c r="J31" s="62">
         <v>2</v>
       </c>
       <c r="K31" s="11">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L31" s="87" t="s">
+      <c r="L31" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M31" s="12">
         <v>0.12</v>
       </c>
-      <c r="N31" s="48">
+      <c r="N31" s="39">
         <f t="shared" si="2"/>
         <v>0.24</v>
       </c>
       <c r="O31" s="12">
         <v>0.10199999999999999</v>
       </c>
-      <c r="P31" s="49">
+      <c r="P31" s="40">
         <f t="shared" si="0"/>
         <v>1.02</v>
       </c>
@@ -3527,47 +3494,47 @@
       <c r="A32" s="16">
         <v>30</v>
       </c>
-      <c r="B32" s="37"/>
-      <c r="C32" s="71" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="71" t="s">
-        <v>104</v>
-      </c>
-      <c r="E32" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F32" s="71" t="s">
-        <v>171</v>
-      </c>
-      <c r="G32" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H32" s="83"/>
-      <c r="I32" s="71" t="s">
-        <v>203</v>
-      </c>
-      <c r="J32" s="72">
+      <c r="B32" s="108"/>
+      <c r="C32" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="D32" s="61" t="s">
+        <v>103</v>
+      </c>
+      <c r="E32" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F32" s="61" t="s">
+        <v>170</v>
+      </c>
+      <c r="G32" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H32" s="73"/>
+      <c r="I32" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="J32" s="62">
         <v>2</v>
       </c>
       <c r="K32" s="11">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L32" s="87" t="s">
+      <c r="L32" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M32" s="12">
         <v>0.1</v>
       </c>
-      <c r="N32" s="48">
+      <c r="N32" s="39">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
       <c r="O32" s="12">
         <v>0.04</v>
       </c>
-      <c r="P32" s="49">
+      <c r="P32" s="40">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
@@ -3577,47 +3544,47 @@
       <c r="A33" s="16">
         <v>31</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="71" t="s">
-        <v>60</v>
-      </c>
-      <c r="D33" s="71" t="s">
-        <v>105</v>
-      </c>
-      <c r="E33" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F33" s="71" t="s">
-        <v>172</v>
-      </c>
-      <c r="G33" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H33" s="83"/>
-      <c r="I33" s="71" t="s">
-        <v>204</v>
-      </c>
-      <c r="J33" s="72">
+      <c r="B33" s="108"/>
+      <c r="C33" s="61" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="61" t="s">
+        <v>104</v>
+      </c>
+      <c r="E33" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" s="61" t="s">
+        <v>171</v>
+      </c>
+      <c r="G33" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H33" s="73"/>
+      <c r="I33" s="61" t="s">
+        <v>203</v>
+      </c>
+      <c r="J33" s="62">
         <v>1</v>
       </c>
       <c r="K33" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L33" s="87" t="s">
+      <c r="L33" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M33" s="12">
         <v>0.1</v>
       </c>
-      <c r="N33" s="48">
+      <c r="N33" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O33" s="12">
         <v>0.1</v>
       </c>
-      <c r="P33" s="49">
+      <c r="P33" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -3627,47 +3594,47 @@
       <c r="A34" s="16">
         <v>32</v>
       </c>
-      <c r="B34" s="37"/>
-      <c r="C34" s="71" t="s">
-        <v>61</v>
-      </c>
-      <c r="D34" s="71" t="s">
-        <v>106</v>
-      </c>
-      <c r="E34" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F34" s="71" t="s">
-        <v>173</v>
-      </c>
-      <c r="G34" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H34" s="83"/>
-      <c r="I34" s="71" t="s">
-        <v>205</v>
-      </c>
-      <c r="J34" s="72">
+      <c r="B34" s="108"/>
+      <c r="C34" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" s="61" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F34" s="61" t="s">
+        <v>172</v>
+      </c>
+      <c r="G34" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H34" s="73"/>
+      <c r="I34" s="61" t="s">
+        <v>204</v>
+      </c>
+      <c r="J34" s="62">
         <v>3</v>
       </c>
       <c r="K34" s="11">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L34" s="87" t="s">
+      <c r="L34" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M34" s="12">
         <v>0.13</v>
       </c>
-      <c r="N34" s="48">
+      <c r="N34" s="39">
         <f t="shared" si="2"/>
         <v>0.39</v>
       </c>
       <c r="O34" s="12">
         <v>0.113</v>
       </c>
-      <c r="P34" s="49">
+      <c r="P34" s="40">
         <f t="shared" si="0"/>
         <v>1.6950000000000001</v>
       </c>
@@ -3677,101 +3644,101 @@
       <c r="A35" s="16">
         <v>33</v>
       </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="71" t="s">
-        <v>62</v>
-      </c>
-      <c r="D35" s="71" t="s">
-        <v>107</v>
-      </c>
-      <c r="E35" s="71" t="s">
-        <v>138</v>
-      </c>
-      <c r="F35" s="71" t="s">
-        <v>174</v>
-      </c>
-      <c r="G35" s="71" t="s">
-        <v>228</v>
-      </c>
-      <c r="H35" s="83" t="s">
-        <v>248</v>
-      </c>
-      <c r="I35" s="71" t="s">
-        <v>206</v>
-      </c>
-      <c r="J35" s="72">
+      <c r="B35" s="108"/>
+      <c r="C35" s="61" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35" s="61" t="s">
+        <v>106</v>
+      </c>
+      <c r="E35" s="61" t="s">
+        <v>137</v>
+      </c>
+      <c r="F35" s="61" t="s">
+        <v>173</v>
+      </c>
+      <c r="G35" s="61" t="s">
+        <v>227</v>
+      </c>
+      <c r="H35" s="73" t="s">
+        <v>247</v>
+      </c>
+      <c r="I35" s="61" t="s">
+        <v>205</v>
+      </c>
+      <c r="J35" s="62">
         <v>1</v>
       </c>
       <c r="K35" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L35" s="87" t="s">
-        <v>249</v>
+      <c r="L35" s="77" t="s">
+        <v>248</v>
       </c>
       <c r="M35" s="12">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="N35" s="48">
+      <c r="N35" s="39">
         <f t="shared" si="2"/>
         <v>8.2000000000000003E-2</v>
       </c>
       <c r="O35" s="12">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="P35" s="49">
+      <c r="P35" s="40">
         <f t="shared" si="0"/>
         <v>0.41000000000000003</v>
       </c>
       <c r="Q35" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="16">
         <v>34</v>
       </c>
-      <c r="B36" s="37"/>
-      <c r="C36" s="71" t="s">
-        <v>57</v>
-      </c>
-      <c r="D36" s="71" t="s">
-        <v>108</v>
-      </c>
-      <c r="E36" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F36" s="71" t="s">
-        <v>169</v>
-      </c>
-      <c r="G36" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H36" s="83"/>
-      <c r="I36" s="71" t="s">
-        <v>27</v>
-      </c>
-      <c r="J36" s="72">
+      <c r="B36" s="108"/>
+      <c r="C36" s="61" t="s">
+        <v>56</v>
+      </c>
+      <c r="D36" s="61" t="s">
+        <v>107</v>
+      </c>
+      <c r="E36" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F36" s="61" t="s">
+        <v>168</v>
+      </c>
+      <c r="G36" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H36" s="73"/>
+      <c r="I36" s="61" t="s">
+        <v>26</v>
+      </c>
+      <c r="J36" s="62">
         <v>4</v>
       </c>
       <c r="K36" s="11">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L36" s="87" t="s">
+      <c r="L36" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M36" s="12">
         <v>0.1</v>
       </c>
-      <c r="N36" s="48">
+      <c r="N36" s="39">
         <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
       <c r="O36" s="12">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="P36" s="49">
+      <c r="P36" s="40">
         <f t="shared" si="0"/>
         <v>0.56000000000000005</v>
       </c>
@@ -3781,47 +3748,47 @@
       <c r="A37" s="16">
         <v>35</v>
       </c>
-      <c r="B37" s="37"/>
-      <c r="C37" s="71" t="s">
-        <v>63</v>
-      </c>
-      <c r="D37" s="71" t="s">
-        <v>109</v>
-      </c>
-      <c r="E37" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F37" s="71" t="s">
-        <v>175</v>
-      </c>
-      <c r="G37" s="71" t="s">
-        <v>216</v>
-      </c>
-      <c r="H37" s="83"/>
-      <c r="I37" s="71" t="s">
-        <v>207</v>
-      </c>
-      <c r="J37" s="72">
+      <c r="B37" s="108"/>
+      <c r="C37" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="D37" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="E37" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" s="61" t="s">
+        <v>174</v>
+      </c>
+      <c r="G37" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="H37" s="73"/>
+      <c r="I37" s="61" t="s">
+        <v>206</v>
+      </c>
+      <c r="J37" s="62">
         <v>1</v>
       </c>
       <c r="K37" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L37" s="87" t="s">
+      <c r="L37" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M37" s="12">
         <v>0.1</v>
       </c>
-      <c r="N37" s="48">
+      <c r="N37" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O37" s="12">
         <v>0.1</v>
       </c>
-      <c r="P37" s="49">
+      <c r="P37" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
@@ -3831,47 +3798,47 @@
       <c r="A38" s="16">
         <v>36</v>
       </c>
-      <c r="B38" s="37"/>
-      <c r="C38" s="71" t="s">
-        <v>64</v>
-      </c>
-      <c r="D38" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="E38" s="71" t="s">
-        <v>139</v>
-      </c>
-      <c r="F38" s="71" t="s">
-        <v>176</v>
-      </c>
-      <c r="G38" s="71"/>
-      <c r="H38" s="83" t="s">
-        <v>252</v>
-      </c>
-      <c r="I38" s="71" t="s">
-        <v>208</v>
-      </c>
-      <c r="J38" s="72">
+      <c r="B38" s="108"/>
+      <c r="C38" s="61" t="s">
+        <v>63</v>
+      </c>
+      <c r="D38" s="61" t="s">
+        <v>109</v>
+      </c>
+      <c r="E38" s="61" t="s">
+        <v>138</v>
+      </c>
+      <c r="F38" s="61" t="s">
+        <v>175</v>
+      </c>
+      <c r="G38" s="61"/>
+      <c r="H38" s="73" t="s">
+        <v>251</v>
+      </c>
+      <c r="I38" s="61" t="s">
+        <v>207</v>
+      </c>
+      <c r="J38" s="62">
         <v>1</v>
       </c>
       <c r="K38" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L38" s="87" t="s">
+      <c r="L38" s="77" t="s">
         <v>23</v>
       </c>
       <c r="M38" s="12">
         <v>0.20100000000000001</v>
       </c>
-      <c r="N38" s="48">
+      <c r="N38" s="39">
         <f t="shared" si="2"/>
         <v>0.20100000000000001</v>
       </c>
       <c r="O38" s="12">
         <v>0.20100000000000001</v>
       </c>
-      <c r="P38" s="49">
+      <c r="P38" s="40">
         <f t="shared" si="0"/>
         <v>1.0050000000000001</v>
       </c>
@@ -3881,247 +3848,247 @@
       <c r="A39" s="16">
         <v>37</v>
       </c>
-      <c r="B39" s="37"/>
-      <c r="C39" s="71" t="s">
-        <v>65</v>
-      </c>
-      <c r="D39" s="71" t="s">
-        <v>111</v>
-      </c>
-      <c r="E39" s="71" t="s">
-        <v>137</v>
-      </c>
-      <c r="F39" s="71" t="s">
-        <v>177</v>
-      </c>
-      <c r="G39" s="71" t="s">
-        <v>226</v>
-      </c>
-      <c r="H39" s="83"/>
-      <c r="I39" s="71" t="s">
-        <v>209</v>
-      </c>
-      <c r="J39" s="72">
+      <c r="B39" s="108"/>
+      <c r="C39" s="61" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" s="61" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="F39" s="61" t="s">
+        <v>176</v>
+      </c>
+      <c r="G39" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="H39" s="73"/>
+      <c r="I39" s="61" t="s">
+        <v>208</v>
+      </c>
+      <c r="J39" s="62">
         <v>1</v>
       </c>
       <c r="K39" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L39" s="87" t="s">
+      <c r="L39" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M39" s="12">
         <v>0.1</v>
       </c>
-      <c r="N39" s="48">
+      <c r="N39" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O39" s="12">
         <v>0.1</v>
       </c>
-      <c r="P39" s="49">
+      <c r="P39" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
       <c r="Q39" s="9"/>
     </row>
     <row r="40" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="32">
+      <c r="A40" s="28">
         <v>38</v>
       </c>
-      <c r="B40" s="39"/>
-      <c r="C40" s="73" t="s">
-        <v>66</v>
-      </c>
-      <c r="D40" s="73" t="s">
-        <v>112</v>
-      </c>
-      <c r="E40" s="73" t="s">
-        <v>137</v>
-      </c>
-      <c r="F40" s="73" t="s">
-        <v>178</v>
-      </c>
-      <c r="G40" s="73" t="s">
-        <v>226</v>
-      </c>
-      <c r="H40" s="84"/>
-      <c r="I40" s="73" t="s">
-        <v>210</v>
-      </c>
-      <c r="J40" s="74">
+      <c r="B40" s="109"/>
+      <c r="C40" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="D40" s="63" t="s">
+        <v>111</v>
+      </c>
+      <c r="E40" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="F40" s="63" t="s">
+        <v>177</v>
+      </c>
+      <c r="G40" s="63" t="s">
+        <v>225</v>
+      </c>
+      <c r="H40" s="74"/>
+      <c r="I40" s="63" t="s">
+        <v>209</v>
+      </c>
+      <c r="J40" s="64">
         <v>1</v>
       </c>
       <c r="K40" s="18">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L40" s="91" t="s">
+      <c r="L40" s="81" t="s">
         <v>14</v>
       </c>
       <c r="M40" s="12">
         <v>0.1</v>
       </c>
-      <c r="N40" s="48">
+      <c r="N40" s="39">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
       <c r="O40" s="12">
         <v>0.1</v>
       </c>
-      <c r="P40" s="49">
+      <c r="P40" s="40">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="Q40" s="34"/>
+      <c r="Q40" s="30"/>
     </row>
     <row r="41" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="50">
+      <c r="A41" s="41">
         <v>39</v>
       </c>
-      <c r="B41" s="104" t="s">
-        <v>242</v>
-      </c>
-      <c r="C41" s="105" t="s">
-        <v>67</v>
-      </c>
-      <c r="D41" s="105" t="s">
-        <v>113</v>
-      </c>
-      <c r="E41" s="105" t="s">
-        <v>140</v>
-      </c>
-      <c r="F41" s="105" t="s">
-        <v>140</v>
-      </c>
-      <c r="G41" s="106"/>
-      <c r="H41" s="107"/>
-      <c r="I41" s="105" t="s">
-        <v>140</v>
-      </c>
-      <c r="J41" s="106">
+      <c r="B41" s="94" t="s">
+        <v>241</v>
+      </c>
+      <c r="C41" s="95" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41" s="95" t="s">
+        <v>112</v>
+      </c>
+      <c r="E41" s="95" t="s">
+        <v>139</v>
+      </c>
+      <c r="F41" s="95" t="s">
+        <v>139</v>
+      </c>
+      <c r="G41" s="96"/>
+      <c r="H41" s="97"/>
+      <c r="I41" s="95" t="s">
+        <v>139</v>
+      </c>
+      <c r="J41" s="96">
         <v>2</v>
       </c>
-      <c r="K41" s="108">
+      <c r="K41" s="98">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L41" s="109" t="s">
+      <c r="L41" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="M41" s="110"/>
-      <c r="N41" s="101">
+      <c r="M41" s="100"/>
+      <c r="N41" s="91">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O41" s="110"/>
-      <c r="P41" s="102">
+      <c r="O41" s="100"/>
+      <c r="P41" s="92">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Q41" s="111"/>
+      <c r="Q41" s="101"/>
     </row>
     <row r="42" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="50">
+      <c r="A42" s="41">
         <v>40</v>
       </c>
-      <c r="B42" s="51" t="s">
-        <v>243</v>
-      </c>
-      <c r="C42" s="75" t="s">
-        <v>68</v>
-      </c>
-      <c r="D42" s="75" t="s">
-        <v>114</v>
-      </c>
-      <c r="E42" s="75" t="s">
-        <v>141</v>
-      </c>
-      <c r="F42" s="75" t="s">
-        <v>141</v>
-      </c>
-      <c r="G42" s="75" t="s">
-        <v>218</v>
-      </c>
-      <c r="H42" s="80"/>
-      <c r="I42" s="75" t="s">
-        <v>141</v>
-      </c>
-      <c r="J42" s="76">
+      <c r="B42" s="42" t="s">
+        <v>242</v>
+      </c>
+      <c r="C42" s="65" t="s">
+        <v>67</v>
+      </c>
+      <c r="D42" s="65" t="s">
+        <v>113</v>
+      </c>
+      <c r="E42" s="65" t="s">
+        <v>140</v>
+      </c>
+      <c r="F42" s="65" t="s">
+        <v>140</v>
+      </c>
+      <c r="G42" s="65" t="s">
+        <v>217</v>
+      </c>
+      <c r="H42" s="70"/>
+      <c r="I42" s="65" t="s">
+        <v>140</v>
+      </c>
+      <c r="J42" s="66">
         <v>1</v>
       </c>
-      <c r="K42" s="52">
+      <c r="K42" s="43">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L42" s="92" t="s">
+      <c r="L42" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="M42" s="53">
+      <c r="M42" s="44">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N42" s="48">
+      <c r="N42" s="39">
         <f t="shared" si="2"/>
         <v>0.55000000000000004</v>
       </c>
-      <c r="O42" s="53">
+      <c r="O42" s="44">
         <v>0.55000000000000004</v>
       </c>
-      <c r="P42" s="49">
+      <c r="P42" s="40">
         <f t="shared" si="0"/>
         <v>2.75</v>
       </c>
-      <c r="Q42" s="54"/>
+      <c r="Q42" s="45"/>
     </row>
     <row r="43" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="22">
         <v>41</v>
       </c>
-      <c r="B43" s="45" t="s">
-        <v>244</v>
-      </c>
-      <c r="C43" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="D43" s="69" t="s">
+      <c r="B43" s="107" t="s">
+        <v>243</v>
+      </c>
+      <c r="C43" s="59" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="E43" s="69" t="s">
-        <v>142</v>
-      </c>
-      <c r="F43" s="69" t="s">
-        <v>142</v>
-      </c>
-      <c r="G43" s="69" t="s">
-        <v>229</v>
-      </c>
-      <c r="H43" s="82"/>
-      <c r="I43" s="69" t="s">
-        <v>142</v>
-      </c>
-      <c r="J43" s="70">
+      <c r="E43" s="59" t="s">
+        <v>141</v>
+      </c>
+      <c r="F43" s="59" t="s">
+        <v>141</v>
+      </c>
+      <c r="G43" s="59" t="s">
+        <v>228</v>
+      </c>
+      <c r="H43" s="72"/>
+      <c r="I43" s="59" t="s">
+        <v>141</v>
+      </c>
+      <c r="J43" s="60">
         <v>1</v>
       </c>
-      <c r="K43" s="46">
+      <c r="K43" s="37">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L43" s="85" t="s">
+      <c r="L43" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="M43" s="47">
+      <c r="M43" s="38">
         <v>3.13</v>
       </c>
-      <c r="N43" s="48">
+      <c r="N43" s="39">
         <f t="shared" si="2"/>
         <v>3.13</v>
       </c>
-      <c r="O43" s="47">
+      <c r="O43" s="38">
         <v>3.13</v>
       </c>
-      <c r="P43" s="49">
+      <c r="P43" s="40">
         <f t="shared" si="0"/>
         <v>15.649999999999999</v>
       </c>
@@ -4131,47 +4098,47 @@
       <c r="A44" s="16">
         <v>42</v>
       </c>
-      <c r="B44" s="37"/>
-      <c r="C44" s="71" t="s">
-        <v>70</v>
-      </c>
-      <c r="D44" s="71" t="s">
-        <v>28</v>
-      </c>
-      <c r="E44" s="71" t="s">
-        <v>143</v>
-      </c>
-      <c r="F44" s="71" t="s">
-        <v>143</v>
-      </c>
-      <c r="G44" s="71" t="s">
-        <v>229</v>
-      </c>
-      <c r="H44" s="83"/>
-      <c r="I44" s="71" t="s">
-        <v>143</v>
-      </c>
-      <c r="J44" s="72">
+      <c r="B44" s="108"/>
+      <c r="C44" s="61" t="s">
+        <v>69</v>
+      </c>
+      <c r="D44" s="61" t="s">
+        <v>27</v>
+      </c>
+      <c r="E44" s="61" t="s">
+        <v>142</v>
+      </c>
+      <c r="F44" s="61" t="s">
+        <v>142</v>
+      </c>
+      <c r="G44" s="61" t="s">
+        <v>228</v>
+      </c>
+      <c r="H44" s="73"/>
+      <c r="I44" s="61" t="s">
+        <v>142</v>
+      </c>
+      <c r="J44" s="62">
         <v>1</v>
       </c>
       <c r="K44" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L44" s="87" t="s">
+      <c r="L44" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M44" s="12">
         <v>1.36</v>
       </c>
-      <c r="N44" s="48">
+      <c r="N44" s="39">
         <f t="shared" si="2"/>
         <v>1.36</v>
       </c>
       <c r="O44" s="12">
         <v>1.36</v>
       </c>
-      <c r="P44" s="49">
+      <c r="P44" s="40">
         <f t="shared" si="0"/>
         <v>6.8000000000000007</v>
       </c>
@@ -4181,47 +4148,47 @@
       <c r="A45" s="16">
         <v>43</v>
       </c>
-      <c r="B45" s="37"/>
-      <c r="C45" s="71" t="s">
-        <v>71</v>
-      </c>
-      <c r="D45" s="71" t="s">
-        <v>115</v>
-      </c>
-      <c r="E45" s="71" t="s">
-        <v>144</v>
-      </c>
-      <c r="F45" s="71" t="s">
-        <v>144</v>
-      </c>
-      <c r="G45" s="71" t="s">
-        <v>230</v>
-      </c>
-      <c r="H45" s="83"/>
-      <c r="I45" s="71" t="s">
-        <v>144</v>
-      </c>
-      <c r="J45" s="72">
+      <c r="B45" s="108"/>
+      <c r="C45" s="61" t="s">
+        <v>70</v>
+      </c>
+      <c r="D45" s="61" t="s">
+        <v>114</v>
+      </c>
+      <c r="E45" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="F45" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="G45" s="61" t="s">
+        <v>229</v>
+      </c>
+      <c r="H45" s="73"/>
+      <c r="I45" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="J45" s="62">
         <v>1</v>
       </c>
       <c r="K45" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L45" s="87" t="s">
+      <c r="L45" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M45" s="12">
         <v>0.54</v>
       </c>
-      <c r="N45" s="48">
+      <c r="N45" s="39">
         <f t="shared" si="2"/>
         <v>0.54</v>
       </c>
       <c r="O45" s="12">
         <v>0.54</v>
       </c>
-      <c r="P45" s="49">
+      <c r="P45" s="40">
         <f t="shared" si="0"/>
         <v>2.7</v>
       </c>
@@ -4231,47 +4198,47 @@
       <c r="A46" s="16">
         <v>44</v>
       </c>
-      <c r="B46" s="37"/>
-      <c r="C46" s="71" t="s">
-        <v>72</v>
-      </c>
-      <c r="D46" s="71" t="s">
-        <v>116</v>
-      </c>
-      <c r="E46" s="71" t="s">
-        <v>145</v>
-      </c>
-      <c r="F46" s="71" t="s">
-        <v>179</v>
-      </c>
-      <c r="G46" s="71" t="s">
-        <v>231</v>
-      </c>
-      <c r="H46" s="83"/>
-      <c r="I46" s="71" t="s">
-        <v>179</v>
-      </c>
-      <c r="J46" s="72">
+      <c r="B46" s="108"/>
+      <c r="C46" s="61" t="s">
+        <v>71</v>
+      </c>
+      <c r="D46" s="61" t="s">
+        <v>115</v>
+      </c>
+      <c r="E46" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="F46" s="61" t="s">
+        <v>178</v>
+      </c>
+      <c r="G46" s="61" t="s">
+        <v>230</v>
+      </c>
+      <c r="H46" s="73"/>
+      <c r="I46" s="61" t="s">
+        <v>178</v>
+      </c>
+      <c r="J46" s="62">
         <v>1</v>
       </c>
       <c r="K46" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L46" s="87" t="s">
+      <c r="L46" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M46" s="12">
         <v>4.5</v>
       </c>
-      <c r="N46" s="48">
+      <c r="N46" s="39">
         <f t="shared" si="2"/>
         <v>4.5</v>
       </c>
       <c r="O46" s="12">
         <v>4.5</v>
       </c>
-      <c r="P46" s="49">
+      <c r="P46" s="40">
         <f t="shared" si="0"/>
         <v>22.5</v>
       </c>
@@ -4281,47 +4248,47 @@
       <c r="A47" s="16">
         <v>45</v>
       </c>
-      <c r="B47" s="37"/>
-      <c r="C47" s="71" t="s">
-        <v>73</v>
-      </c>
-      <c r="D47" s="71" t="s">
-        <v>117</v>
-      </c>
-      <c r="E47" s="71" t="s">
-        <v>146</v>
-      </c>
-      <c r="F47" s="71" t="s">
-        <v>180</v>
-      </c>
-      <c r="G47" s="71" t="s">
-        <v>232</v>
-      </c>
-      <c r="H47" s="83"/>
-      <c r="I47" s="71" t="s">
-        <v>211</v>
-      </c>
-      <c r="J47" s="72">
+      <c r="B47" s="108"/>
+      <c r="C47" s="61" t="s">
+        <v>72</v>
+      </c>
+      <c r="D47" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="E47" s="61" t="s">
+        <v>145</v>
+      </c>
+      <c r="F47" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="G47" s="61" t="s">
+        <v>231</v>
+      </c>
+      <c r="H47" s="73"/>
+      <c r="I47" s="61" t="s">
+        <v>210</v>
+      </c>
+      <c r="J47" s="62">
         <v>1</v>
       </c>
       <c r="K47" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L47" s="87" t="s">
+      <c r="L47" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M47" s="12">
         <v>2.74</v>
       </c>
-      <c r="N47" s="48">
+      <c r="N47" s="39">
         <f t="shared" si="2"/>
         <v>2.74</v>
       </c>
       <c r="O47" s="12">
         <v>2.74</v>
       </c>
-      <c r="P47" s="49">
+      <c r="P47" s="40">
         <f t="shared" si="0"/>
         <v>13.700000000000001</v>
       </c>
@@ -4331,174 +4298,174 @@
       <c r="A48" s="16">
         <v>46</v>
       </c>
-      <c r="B48" s="37"/>
-      <c r="C48" s="71" t="s">
-        <v>74</v>
-      </c>
-      <c r="D48" s="71" t="s">
-        <v>118</v>
-      </c>
-      <c r="E48" s="71" t="s">
-        <v>147</v>
-      </c>
-      <c r="F48" s="71" t="s">
-        <v>181</v>
-      </c>
-      <c r="G48" s="72"/>
-      <c r="H48" s="83"/>
-      <c r="I48" s="71" t="s">
-        <v>181</v>
-      </c>
-      <c r="J48" s="72">
+      <c r="B48" s="108"/>
+      <c r="C48" s="61" t="s">
+        <v>73</v>
+      </c>
+      <c r="D48" s="61" t="s">
+        <v>117</v>
+      </c>
+      <c r="E48" s="61" t="s">
+        <v>146</v>
+      </c>
+      <c r="F48" s="61" t="s">
+        <v>180</v>
+      </c>
+      <c r="G48" s="62"/>
+      <c r="H48" s="73"/>
+      <c r="I48" s="61" t="s">
+        <v>180</v>
+      </c>
+      <c r="J48" s="62">
         <v>1</v>
       </c>
       <c r="K48" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L48" s="87" t="s">
-        <v>251</v>
+      <c r="L48" s="77" t="s">
+        <v>250</v>
       </c>
       <c r="M48" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="N48" s="48" t="e">
+        <v>24</v>
+      </c>
+      <c r="N48" s="39" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
       <c r="O48" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="P48" s="49">
+        <v>24</v>
+      </c>
+      <c r="P48" s="40">
         <v>7.34</v>
       </c>
       <c r="Q48" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="49" spans="1:17" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="32">
+      <c r="A49" s="28">
         <v>47</v>
       </c>
-      <c r="B49" s="39"/>
-      <c r="C49" s="73" t="s">
-        <v>76</v>
-      </c>
-      <c r="D49" s="73" t="s">
-        <v>120</v>
-      </c>
-      <c r="E49" s="73" t="s">
-        <v>147</v>
-      </c>
-      <c r="F49" s="73" t="s">
-        <v>182</v>
-      </c>
-      <c r="G49" s="73" t="s">
-        <v>234</v>
-      </c>
-      <c r="H49" s="84"/>
-      <c r="I49" s="73" t="s">
-        <v>182</v>
-      </c>
-      <c r="J49" s="74">
+      <c r="B49" s="109"/>
+      <c r="C49" s="63" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49" s="63" t="s">
+        <v>119</v>
+      </c>
+      <c r="E49" s="63" t="s">
+        <v>146</v>
+      </c>
+      <c r="F49" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="G49" s="63" t="s">
+        <v>233</v>
+      </c>
+      <c r="H49" s="74"/>
+      <c r="I49" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="J49" s="64">
         <v>1</v>
       </c>
       <c r="K49" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L49" s="87" t="s">
-        <v>251</v>
+      <c r="L49" s="77" t="s">
+        <v>250</v>
       </c>
       <c r="M49" s="20">
         <v>0.71</v>
       </c>
-      <c r="N49" s="48">
+      <c r="N49" s="39">
         <f t="shared" si="2"/>
         <v>0.71</v>
       </c>
       <c r="O49" s="20">
         <v>0.71</v>
       </c>
-      <c r="P49" s="49">
+      <c r="P49" s="40">
         <f t="shared" si="0"/>
         <v>3.55</v>
       </c>
-      <c r="Q49" s="34"/>
+      <c r="Q49" s="30"/>
     </row>
     <row r="50" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="22">
         <v>48</v>
       </c>
-      <c r="B50" s="42" t="s">
-        <v>245</v>
-      </c>
-      <c r="C50" s="71" t="s">
-        <v>75</v>
-      </c>
-      <c r="D50" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="E50" s="71" t="s">
-        <v>148</v>
-      </c>
-      <c r="F50" s="71" t="s">
-        <v>148</v>
-      </c>
-      <c r="G50" s="71" t="s">
-        <v>233</v>
-      </c>
-      <c r="H50" s="83"/>
-      <c r="I50" s="71" t="s">
-        <v>148</v>
-      </c>
-      <c r="J50" s="72">
+      <c r="B50" s="34" t="s">
+        <v>244</v>
+      </c>
+      <c r="C50" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="D50" s="61" t="s">
+        <v>118</v>
+      </c>
+      <c r="E50" s="61" t="s">
+        <v>147</v>
+      </c>
+      <c r="F50" s="61" t="s">
+        <v>147</v>
+      </c>
+      <c r="G50" s="61" t="s">
+        <v>232</v>
+      </c>
+      <c r="H50" s="73"/>
+      <c r="I50" s="61" t="s">
+        <v>147</v>
+      </c>
+      <c r="J50" s="62">
         <v>1</v>
       </c>
       <c r="K50" s="11">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L50" s="87" t="s">
+      <c r="L50" s="77" t="s">
         <v>14</v>
       </c>
       <c r="M50" s="12">
         <v>0.73</v>
       </c>
-      <c r="N50" s="48">
+      <c r="N50" s="39">
         <f t="shared" si="2"/>
         <v>0.73</v>
       </c>
       <c r="O50" s="12">
         <v>0.73</v>
       </c>
-      <c r="P50" s="49">
+      <c r="P50" s="40">
         <f t="shared" si="0"/>
         <v>3.65</v>
       </c>
       <c r="Q50" s="9"/>
     </row>
     <row r="51" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="44"/>
-      <c r="B51" s="43"/>
-      <c r="C51" s="73"/>
-      <c r="D51" s="73"/>
-      <c r="E51" s="73"/>
-      <c r="F51" s="73"/>
-      <c r="G51" s="73"/>
-      <c r="H51" s="84"/>
-      <c r="I51" s="73"/>
-      <c r="J51" s="74"/>
+      <c r="A51" s="36"/>
+      <c r="B51" s="35"/>
+      <c r="C51" s="63"/>
+      <c r="D51" s="63"/>
+      <c r="E51" s="63"/>
+      <c r="F51" s="63"/>
+      <c r="G51" s="63"/>
+      <c r="H51" s="74"/>
+      <c r="I51" s="63"/>
+      <c r="J51" s="64"/>
       <c r="K51" s="18"/>
       <c r="L51" s="19"/>
       <c r="M51" s="20"/>
       <c r="N51" s="21"/>
-      <c r="O51" s="33"/>
-      <c r="P51" s="49"/>
-      <c r="Q51" s="34"/>
+      <c r="O51" s="29"/>
+      <c r="P51" s="40"/>
+      <c r="Q51" s="30"/>
     </row>
     <row r="52" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="41"/>
+      <c r="A52" s="33"/>
       <c r="B52"/>
       <c r="C52"/>
       <c r="D52"/>
@@ -4507,22 +4474,22 @@
       <c r="G52"/>
       <c r="H52"/>
       <c r="I52"/>
-      <c r="J52" s="28" t="s">
+      <c r="J52" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="K52" s="28"/>
-      <c r="L52" s="28"/>
-      <c r="M52" s="28"/>
+      <c r="K52" s="106"/>
+      <c r="L52" s="106"/>
+      <c r="M52" s="106"/>
       <c r="N52" s="2"/>
       <c r="O52" s="3"/>
       <c r="P52" s="3">
         <f>SUM(P3:P21)</f>
         <v>46.304000000000009</v>
       </c>
-      <c r="Q52" s="29"/>
+      <c r="Q52" s="25"/>
     </row>
     <row r="53" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="32"/>
+      <c r="A53" s="28"/>
       <c r="B53"/>
       <c r="C53"/>
       <c r="D53"/>
@@ -4531,12 +4498,12 @@
       <c r="G53"/>
       <c r="H53"/>
       <c r="I53"/>
-      <c r="J53" s="25" t="s">
+      <c r="J53" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="K53" s="25"/>
-      <c r="L53" s="25"/>
-      <c r="M53" s="25"/>
+      <c r="K53" s="102"/>
+      <c r="L53" s="102"/>
+      <c r="M53" s="102"/>
       <c r="N53" s="4">
         <f>SUM(N3:N21)</f>
         <v>11.670999999999999</v>
@@ -4599,7 +4566,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q3:Q48 Q50:Q51">
+  <conditionalFormatting sqref="Q50:Q51 Q3:Q48">
     <cfRule type="dataBar" priority="49">
       <dataBar>
         <cfvo type="min"/>
@@ -4642,51 +4609,51 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="L3" r:id="rId1" xr:uid="{761F341B-C913-433E-A082-E7D93AB0DD81}"/>
-    <hyperlink ref="L4" r:id="rId2" xr:uid="{67D49F67-9FCB-40BE-BACC-FC8B21A4CC5B}"/>
-    <hyperlink ref="L5" r:id="rId3" xr:uid="{B62E8DC4-C315-4E04-860F-BB51A258BC25}"/>
-    <hyperlink ref="L6" r:id="rId4" xr:uid="{DC9014C7-4741-4C4C-8DE1-CB0206574EFB}"/>
-    <hyperlink ref="L7" r:id="rId5" xr:uid="{D480674F-F807-437D-A5A9-20B5370707B1}"/>
-    <hyperlink ref="L8" r:id="rId6" xr:uid="{DCBF9CC7-B13A-473D-AA62-A9C1938F80D7}"/>
-    <hyperlink ref="L9" r:id="rId7" xr:uid="{06A219AF-8CFB-44CD-880C-B02B25878119}"/>
-    <hyperlink ref="L10" r:id="rId8" xr:uid="{E267CE76-5124-4196-8850-9C8D89B82D83}"/>
-    <hyperlink ref="L11" r:id="rId9" xr:uid="{E6CECBD2-8E3B-4A63-BD3F-D765DCF3EE80}"/>
-    <hyperlink ref="L12" r:id="rId10" xr:uid="{FC843216-D495-4CB5-A656-277C003D353A}"/>
-    <hyperlink ref="L13" r:id="rId11" xr:uid="{EF80E1E6-5D1C-45AA-8D21-499109B992E7}"/>
-    <hyperlink ref="L14" r:id="rId12" xr:uid="{48FBA434-CB54-4115-B046-AE18C1211EFD}"/>
-    <hyperlink ref="L15" r:id="rId13" xr:uid="{948BB74F-A582-4FEC-937C-9C7DD215F983}"/>
-    <hyperlink ref="L18" r:id="rId14" xr:uid="{47C2C492-0E88-469D-99B2-5D3E4E29E6B9}"/>
-    <hyperlink ref="L19" r:id="rId15" xr:uid="{8DA18EAB-1386-4B1F-85D7-D1E8A143C02F}"/>
-    <hyperlink ref="L20" r:id="rId16" xr:uid="{6A5EED19-9CCB-4CB6-8DB2-9D7FC1594963}"/>
-    <hyperlink ref="L21" r:id="rId17" xr:uid="{DCFB836D-AA32-45F9-B42F-95A6AD595F3B}"/>
-    <hyperlink ref="L22" r:id="rId18" xr:uid="{F1C16BC1-6114-42EA-8796-8EB0CADDDF7E}"/>
-    <hyperlink ref="L23" r:id="rId19" xr:uid="{1E5E97B3-7A91-4EE5-BAC1-5A6D39EC2C92}"/>
-    <hyperlink ref="L24" r:id="rId20" xr:uid="{45C8C639-71C2-4D40-B25C-D70E38A875E5}"/>
-    <hyperlink ref="L25" r:id="rId21" xr:uid="{47A52AD3-30A6-463E-8534-E6A044756697}"/>
-    <hyperlink ref="L26" r:id="rId22" xr:uid="{6042D158-D60D-4806-AFFB-0F7F388C29A9}"/>
-    <hyperlink ref="L27" r:id="rId23" xr:uid="{E02F0075-ADDB-4504-AF5C-6C04C094C30D}"/>
-    <hyperlink ref="L28" r:id="rId24" xr:uid="{896515EB-F9C2-44F2-BDA9-04334889FD25}"/>
-    <hyperlink ref="L29" r:id="rId25" xr:uid="{A81927B5-8707-4B7E-ACEB-473A94732F7C}"/>
-    <hyperlink ref="L30" r:id="rId26" xr:uid="{D9683887-9877-4E0C-B567-C081D41F94E9}"/>
-    <hyperlink ref="L31" r:id="rId27" xr:uid="{B43EF50D-C055-4345-899F-22ECBEA18F2B}"/>
-    <hyperlink ref="L32" r:id="rId28" xr:uid="{3B3E03B7-EBB9-4AD7-9D40-CA1DA622FDC7}"/>
-    <hyperlink ref="L33" r:id="rId29" xr:uid="{A9E201B3-E729-44F4-B024-0CE2857AB436}"/>
-    <hyperlink ref="L34" r:id="rId30" xr:uid="{481647A9-8070-4492-AFC8-76654F920BAE}"/>
-    <hyperlink ref="L35" r:id="rId31" xr:uid="{BC835B7C-00C3-4CD7-B18A-3FD6D1FE090E}"/>
-    <hyperlink ref="L36" r:id="rId32" xr:uid="{13702011-3B2A-4CE5-9347-64E93055391C}"/>
-    <hyperlink ref="L37" r:id="rId33" xr:uid="{1138333D-0F0F-49E2-9DD5-986C36956FC1}"/>
-    <hyperlink ref="L38" r:id="rId34" xr:uid="{8D90F7AF-3FE7-49DC-9A25-887D6B56749E}"/>
-    <hyperlink ref="L39" r:id="rId35" xr:uid="{03CBD172-3C95-41A5-9505-12F8046FAC1C}"/>
-    <hyperlink ref="L40" r:id="rId36" xr:uid="{5A3A5E3F-A2D1-46A1-8D54-336D5602B8C3}"/>
-    <hyperlink ref="L42" r:id="rId37" xr:uid="{659858BE-7749-4B20-8A26-A4496C893C8B}"/>
-    <hyperlink ref="L43" r:id="rId38" xr:uid="{46D24381-0767-4D74-A865-7B39430FBA38}"/>
-    <hyperlink ref="L44" r:id="rId39" xr:uid="{BB1F4151-250A-4CDD-B7BA-C78D6DAFAA68}"/>
-    <hyperlink ref="L45" r:id="rId40" xr:uid="{DA3C0E1E-8DA3-4948-94C5-B4E44CFC3BE8}"/>
-    <hyperlink ref="L46" r:id="rId41" xr:uid="{AA867F72-54F4-4956-9629-CE58DC1B4960}"/>
-    <hyperlink ref="L47" r:id="rId42" xr:uid="{886F3C25-32AD-4FDD-82B8-F6C91C1148FF}"/>
-    <hyperlink ref="L50" r:id="rId43" xr:uid="{0E9DCD41-1615-45FB-9260-6D4DD5B433DD}"/>
-    <hyperlink ref="L48" r:id="rId44" xr:uid="{9A306BC8-F47C-404D-B220-008F20D3ECF7}"/>
-    <hyperlink ref="L49" r:id="rId45" xr:uid="{E3289C0C-726F-4E62-A519-870FB919F7EC}"/>
+    <hyperlink ref="L3" r:id="rId1"/>
+    <hyperlink ref="L4" r:id="rId2"/>
+    <hyperlink ref="L5" r:id="rId3"/>
+    <hyperlink ref="L6" r:id="rId4"/>
+    <hyperlink ref="L7" r:id="rId5"/>
+    <hyperlink ref="L8" r:id="rId6"/>
+    <hyperlink ref="L9" r:id="rId7"/>
+    <hyperlink ref="L10" r:id="rId8"/>
+    <hyperlink ref="L11" r:id="rId9"/>
+    <hyperlink ref="L12" r:id="rId10"/>
+    <hyperlink ref="L13" r:id="rId11"/>
+    <hyperlink ref="L14" r:id="rId12"/>
+    <hyperlink ref="L15" r:id="rId13"/>
+    <hyperlink ref="L18" r:id="rId14"/>
+    <hyperlink ref="L19" r:id="rId15"/>
+    <hyperlink ref="L20" r:id="rId16"/>
+    <hyperlink ref="L21" r:id="rId17"/>
+    <hyperlink ref="L22" r:id="rId18"/>
+    <hyperlink ref="L23" r:id="rId19"/>
+    <hyperlink ref="L24" r:id="rId20"/>
+    <hyperlink ref="L25" r:id="rId21"/>
+    <hyperlink ref="L26" r:id="rId22"/>
+    <hyperlink ref="L27" r:id="rId23"/>
+    <hyperlink ref="L28" r:id="rId24"/>
+    <hyperlink ref="L29" r:id="rId25"/>
+    <hyperlink ref="L30" r:id="rId26"/>
+    <hyperlink ref="L31" r:id="rId27"/>
+    <hyperlink ref="L32" r:id="rId28"/>
+    <hyperlink ref="L33" r:id="rId29"/>
+    <hyperlink ref="L34" r:id="rId30"/>
+    <hyperlink ref="L35" r:id="rId31"/>
+    <hyperlink ref="L36" r:id="rId32"/>
+    <hyperlink ref="L37" r:id="rId33"/>
+    <hyperlink ref="L38" r:id="rId34"/>
+    <hyperlink ref="L39" r:id="rId35"/>
+    <hyperlink ref="L40" r:id="rId36"/>
+    <hyperlink ref="L42" r:id="rId37"/>
+    <hyperlink ref="L43" r:id="rId38"/>
+    <hyperlink ref="L44" r:id="rId39"/>
+    <hyperlink ref="L45" r:id="rId40"/>
+    <hyperlink ref="L46" r:id="rId41"/>
+    <hyperlink ref="L47" r:id="rId42"/>
+    <hyperlink ref="L50" r:id="rId43"/>
+    <hyperlink ref="L48" r:id="rId44"/>
+    <hyperlink ref="L49" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId46"/>
@@ -4730,7 +4697,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>Q3:Q48 Q50:Q51</xm:sqref>
+          <xm:sqref>Q50:Q51 Q3:Q48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{9F41C311-B53F-4FDE-A999-535E1BB8B4D8}">

</xml_diff>